<commit_message>
fix: refresh frontend assets for August filter
</commit_message>
<xml_diff>
--- a/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
+++ b/Planilhas/MONITORAMENTOS DE ALARMES COORDENACAO COR ABRIL-junho26 (consolidado).xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Repo\Ocorrencias_Espontaneas\Planilhas\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{34DAD0B4-324E-45EB-8049-3536265DCF36}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5835992C-D678-4934-B269-1D67EF746BA6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-28920" yWindow="525" windowWidth="29040" windowHeight="15720" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9382" uniqueCount="2938">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9384" uniqueCount="2939">
   <si>
     <t>Data</t>
   </si>
@@ -8855,6 +8855,9 @@
   </si>
   <si>
     <t>BOULEVARD VINTE E OITO DE SETEMBRO - VILA ISABEL - ALT. Nº 277</t>
+  </si>
+  <si>
+    <t>AGOSTO</t>
   </si>
 </sst>
 </file>
@@ -8865,7 +8868,7 @@
     <numFmt numFmtId="164" formatCode="d/mmm"/>
     <numFmt numFmtId="165" formatCode="d\-mmm"/>
   </numFmts>
-  <fonts count="25">
+  <fonts count="26">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -9008,6 +9011,11 @@
       <sz val="8"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -9600,7 +9608,9 @@
       <c r="M3" s="3" t="s">
         <v>2141</v>
       </c>
-      <c r="N3" s="2"/>
+      <c r="N3" s="3" t="s">
+        <v>2938</v>
+      </c>
       <c r="O3" s="2"/>
       <c r="P3" s="2"/>
       <c r="Q3" s="2"/>
@@ -9641,7 +9651,9 @@
       <c r="M4" s="9">
         <v>2530</v>
       </c>
-      <c r="N4" s="4"/>
+      <c r="N4" s="9">
+        <v>2470</v>
+      </c>
       <c r="O4" s="4"/>
       <c r="P4" s="4"/>
       <c r="Q4" s="4"/>
@@ -9686,7 +9698,9 @@
       <c r="M5" s="9">
         <v>367</v>
       </c>
-      <c r="N5" s="10"/>
+      <c r="N5" s="9">
+        <v>504</v>
+      </c>
       <c r="O5" s="10"/>
       <c r="P5" s="10"/>
       <c r="Q5" s="10"/>
@@ -9799,7 +9813,9 @@
       <c r="M8" s="3" t="s">
         <v>2141</v>
       </c>
-      <c r="N8" s="9"/>
+      <c r="N8" s="3" t="s">
+        <v>2938</v>
+      </c>
       <c r="O8" s="9"/>
       <c r="P8" s="9"/>
       <c r="Q8" s="9"/>
@@ -9849,7 +9865,10 @@
         <f>100%-M10</f>
         <v>0.85494071146245054</v>
       </c>
-      <c r="N9" s="9"/>
+      <c r="N9" s="16">
+        <f>100%-N10</f>
+        <v>0.79595141700404859</v>
+      </c>
       <c r="O9" s="9"/>
       <c r="P9" s="9"/>
       <c r="Q9" s="9"/>
@@ -9897,7 +9916,10 @@
         <f>M5/M4</f>
         <v>0.1450592885375494</v>
       </c>
-      <c r="N10" s="9"/>
+      <c r="N10" s="16">
+        <f>N5/N4</f>
+        <v>0.20404858299595141</v>
+      </c>
       <c r="O10" s="9"/>
       <c r="P10" s="9"/>
       <c r="Q10" s="9"/>
@@ -50411,6 +50433,7 @@
       </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="25" type="noConversion"/>
   <pageMargins left="0.51180555555555596" right="0.51180555555555596" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup orientation="landscape" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>

</xml_diff>